<commit_message>
Remove financial KPI from Corp Planning goal-setting sheet
Corp Planning sets non-financial KPIs only, so L6 now uses the same
70% competency / 30% non-financial KPI split as L4-L5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rijr1SmZgUsjydfrH97SCU
</commit_message>
<xml_diff>
--- a/FY27_CorpPlanning_目標設定シート_v0.1.xlsx
+++ b/FY27_CorpPlanning_目標設定シート_v0.1.xlsx
@@ -414,7 +414,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="366">
   <si>
     <r>
       <rPr>
@@ -5011,55 +5011,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">非財務</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI 30%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・財務</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI 20%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（評価全体）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
         <rFont val="WenQuanYi Zen Hei"/>
@@ -5198,7 +5149,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">目標とコンピテンシー評価の比率はコンピテンシー定義書 </t>
+      <t xml:space="preserve">目標は</t>
     </r>
     <r>
       <rPr>
@@ -5208,7 +5159,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Ver.0.14.3</t>
+      <t xml:space="preserve">L4</t>
     </r>
     <r>
       <rPr>
@@ -5217,7 +5168,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">（</t>
+      <t xml:space="preserve">以上の非財務</t>
     </r>
     <r>
       <rPr>
@@ -5227,7 +5178,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">M</t>
+      <t xml:space="preserve">KPI</t>
     </r>
     <r>
       <rPr>
@@ -5236,7 +5187,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">・</t>
+      <t xml:space="preserve">のみ（</t>
     </r>
     <r>
       <rPr>
@@ -5246,7 +5197,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">SM</t>
+      <t xml:space="preserve">Corp Planning</t>
     </r>
     <r>
       <rPr>
@@ -5255,7 +5206,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">＝</t>
+      <t xml:space="preserve">では財務</t>
     </r>
     <r>
       <rPr>
@@ -5265,7 +5216,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">L4</t>
+      <t xml:space="preserve">KPI</t>
     </r>
     <r>
       <rPr>
@@ -5274,7 +5225,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">〜</t>
+      <t xml:space="preserve">は設定しない）。比率はコンピテンシー</t>
     </r>
     <r>
       <rPr>
@@ -5284,7 +5235,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">L5</t>
+      <t xml:space="preserve">70%</t>
     </r>
     <r>
       <rPr>
@@ -5293,7 +5244,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">、</t>
+      <t xml:space="preserve">・非財務</t>
     </r>
     <r>
       <rPr>
@@ -5303,7 +5254,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">D</t>
+      <t xml:space="preserve">KPI 30%</t>
     </r>
     <r>
       <rPr>
@@ -5312,7 +5263,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">・</t>
+      <t xml:space="preserve">（定義書 </t>
     </r>
     <r>
       <rPr>
@@ -5322,7 +5273,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">MD</t>
+      <t xml:space="preserve">Ver.0.14.3</t>
     </r>
     <r>
       <rPr>
@@ -5331,7 +5282,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">＝</t>
+      <t xml:space="preserve">の</t>
     </r>
     <r>
       <rPr>
@@ -5341,7 +5292,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">L6</t>
+      <t xml:space="preserve">M</t>
     </r>
     <r>
       <rPr>
@@ -5350,67 +5301,67 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">として仮置き）。</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">・</t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">出所：</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SM</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CorpPlanning_</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の比率を</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">タイトル別コンピテンシー定義</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L4</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ドラフト</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L6</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">_v02</t>
-    </r>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">に適用）。</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="9"/>
@@ -5418,7 +5369,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">「レベル別の評価ウェイト」。</t>
+      <t xml:space="preserve">出所：</t>
     </r>
     <r>
       <rPr>
@@ -5428,7 +5379,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">L1</t>
+      <t xml:space="preserve">CorpPlanning_</t>
     </r>
     <r>
       <rPr>
@@ -5437,7 +5388,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">〜</t>
+      <t xml:space="preserve">タイトル別コンピテンシー定義</t>
     </r>
     <r>
       <rPr>
@@ -5447,7 +5398,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">L3</t>
+      <t xml:space="preserve">_</t>
     </r>
     <r>
       <rPr>
@@ -5456,7 +5407,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">は現行</t>
+      <t xml:space="preserve">ドラフト</t>
     </r>
     <r>
       <rPr>
@@ -5466,7 +5417,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Junior</t>
+      <t xml:space="preserve">_v02</t>
     </r>
     <r>
       <rPr>
@@ -5475,507 +5426,507 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">評価シートのウェイトに統一。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L1 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">スタッフ／サブチーフ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L2 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">チーフ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L3 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">アシスタントマネジャー／デピュティマネジャー</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L4 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">マネジャー</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L5 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">アソシエイトディレクター／デピュティディレクター</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L6 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ディレクター</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">上長の支援で課題を整理する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">自ら仮説を立てて構造化する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">担当領域の課題を自律的に分析する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">複数領域の論点設定・分析をリードする</t>
-  </si>
-  <si>
-    <t xml:space="preserve">部門横断の課題の打ち手を設計する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経営アジェンダの論点設定・提言を行う</t>
-  </si>
-  <si>
-    <t xml:space="preserve">支援を受け期日・品質を守る</t>
-  </si>
-  <si>
-    <t xml:space="preserve">逆算で計画し進捗を自発的に共有する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">担当領域の計画と後輩の進捗を管理する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">複数領域の計画・予算・品質を管理する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">全体のリソース配分を最適化する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経営計画と整合した予算・体制を決定する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">報・連・相を確実に行う</t>
-  </si>
-  <si>
-    <t xml:space="preserve">結論から簡潔に伝える</t>
-  </si>
-  <si>
-    <t xml:space="preserve">多人数の会議をファシリテートする</t>
-  </si>
-  <si>
-    <t xml:space="preserve">事業部門・本体と合意形成する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">対立テーマでも合意形成を主導する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経営会議で意思決定を主導する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">指示どおり正確に作成する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">要点を先に示す簡潔な文書を作る</t>
-  </si>
-  <si>
-    <t xml:space="preserve">意思決定に使える規程・資料を作る</t>
-  </si>
-  <si>
-    <t xml:space="preserve">チームの成果物の品質に責任を持つ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経営向けの方針書・制度案を作成する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">全社・グループへ方針を発信する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">－（育成目標で管理）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">主担当領域で市場水準の専門性を持つ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">複数領域に精通し制度を設計する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">バックオフィス全般で経営に提言する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">フィードバックを受け改善する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">自ら成長目標を設定し学ぶ</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〜</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">L2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">OJT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・業務指導を行う</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">メンバーの育成計画・キャリア支援を行う</t>
-  </si>
-  <si>
-    <t xml:space="preserve">人材要件の定義と採用・育成計画を作る</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Corp Planning</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の人材方針を策定する</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">指示の範囲で協力する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">本体の担当者と自ら連携する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">担当領域の窓口として調整する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">部門責任者と協働環境を整える</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本体・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ICBP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">との連携体制を構築する</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">経営層・グループと信頼関係を構築する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ルールを理解し実践する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">運用する側として改善を提案する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">担当領域の改善・ナレッジ化を進める</t>
-  </si>
-  <si>
-    <t xml:space="preserve">チームの品質・法令順守に責任を持つ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">品質・リスク管理の仕組みを整備する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">カルチャー・リスク文化を醸成する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">精度・期限を守り完遂する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">上長の確認が不要な精度で作成する</t>
-  </si>
-  <si>
-    <t xml:space="preserve">レポート品質とデータ整合を担保する</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">経営資料の品質・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">整合を管理する</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">体系・計画プロセスを設計する</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">経営の意思決定速度に直接貢献する</t>
-  </si>
-  <si>
+      <t xml:space="preserve">「レベル別の評価ウェイト」。</t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">出所：同ドラフト </t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L1</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">v02</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">「コンピテンシー定義（期待水準の要約）」。全文は</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L3</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Excel</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">は現行</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の「</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Junior</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">02_</t>
-    </r>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">評価シートのウェイトに統一。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">スタッフ／サブチーフ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">チーフ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L3 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">アシスタントマネジャー／デピュティマネジャー</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L4 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">マネジャー</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L5 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">アソシエイトディレクター／デピュティディレクター</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L6 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ディレクター</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">上長の支援で課題を整理する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">自ら仮説を立てて構造化する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">担当領域の課題を自律的に分析する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">複数領域の論点設定・分析をリードする</t>
+  </si>
+  <si>
+    <t xml:space="preserve">部門横断の課題の打ち手を設計する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経営アジェンダの論点設定・提言を行う</t>
+  </si>
+  <si>
+    <t xml:space="preserve">支援を受け期日・品質を守る</t>
+  </si>
+  <si>
+    <t xml:space="preserve">逆算で計画し進捗を自発的に共有する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">担当領域の計画と後輩の進捗を管理する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">複数領域の計画・予算・品質を管理する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">全体のリソース配分を最適化する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経営計画と整合した予算・体制を決定する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">報・連・相を確実に行う</t>
+  </si>
+  <si>
+    <t xml:space="preserve">結論から簡潔に伝える</t>
+  </si>
+  <si>
+    <t xml:space="preserve">多人数の会議をファシリテートする</t>
+  </si>
+  <si>
+    <t xml:space="preserve">事業部門・本体と合意形成する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">対立テーマでも合意形成を主導する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経営会議で意思決定を主導する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">指示どおり正確に作成する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">要点を先に示す簡潔な文書を作る</t>
+  </si>
+  <si>
+    <t xml:space="preserve">意思決定に使える規程・資料を作る</t>
+  </si>
+  <si>
+    <t xml:space="preserve">チームの成果物の品質に責任を持つ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経営向けの方針書・制度案を作成する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">全社・グループへ方針を発信する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">－（育成目標で管理）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">主担当領域で市場水準の専門性を持つ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">複数領域に精通し制度を設計する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">バックオフィス全般で経営に提言する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">フィードバックを受け改善する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">自ら成長目標を設定し学ぶ</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">L2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">OJT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・業務指導を行う</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">メンバーの育成計画・キャリア支援を行う</t>
+  </si>
+  <si>
+    <t xml:space="preserve">人材要件の定義と採用・育成計画を作る</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Corp Planning</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の人材方針を策定する</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">指示の範囲で協力する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">本体の担当者と自ら連携する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">担当領域の窓口として調整する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">部門責任者と協働環境を整える</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本体・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ICBP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">との連携体制を構築する</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">経営層・グループと信頼関係を構築する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ルールを理解し実践する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">運用する側として改善を提案する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">担当領域の改善・ナレッジ化を進める</t>
+  </si>
+  <si>
+    <t xml:space="preserve">チームの品質・法令順守に責任を持つ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">品質・リスク管理の仕組みを整備する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">カルチャー・リスク文化を醸成する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">精度・期限を守り完遂する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">上長の確認が不要な精度で作成する</t>
+  </si>
+  <si>
+    <t xml:space="preserve">レポート品質とデータ整合を担保する</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">経営資料の品質・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">KPI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">整合を管理する</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">KPI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">体系・計画プロセスを設計する</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">経営の意思決定速度に直接貢献する</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="9"/>
@@ -5983,584 +5934,584 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">コンピテンシー定義」を参照。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">専門領域</t>
-  </si>
-  <si>
-    <t xml:space="preserve">タイトルに付ける機能名（仮）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">入退社・勤怠・社保の手続</t>
-  </si>
-  <si>
-    <t xml:space="preserve">労務運用・評価の事務局</t>
-  </si>
-  <si>
-    <t xml:space="preserve">運用設計・規程改定の起案</t>
-  </si>
-  <si>
-    <t xml:space="preserve">評価・採用・育成の統括</t>
-  </si>
-  <si>
-    <t xml:space="preserve">要員計画・人事制度の設計</t>
-  </si>
-  <si>
-    <t xml:space="preserve">人事戦略・報酬原資の決定</t>
-  </si>
-  <si>
-    <t xml:space="preserve">総務</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">備品・施設の依頼を処理</t>
-  </si>
-  <si>
-    <t xml:space="preserve">総務運用・社内イベント運営</t>
-  </si>
-  <si>
-    <t xml:space="preserve">総務プロセス設計・ベンダー管理</t>
-  </si>
-  <si>
-    <t xml:space="preserve">総務・規程・監査対応の統括</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">BCP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・リスク管理方針の策定</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">リスク・コンプラ統制の責任者</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経理・財務</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経費精算・請求書のチェック</t>
-  </si>
-  <si>
-    <t xml:space="preserve">計数集計・本体経理との照合</t>
-  </si>
-  <si>
-    <t xml:space="preserve">月次決算・予実分析のリード</t>
-  </si>
-  <si>
-    <t xml:space="preserve">予算・予実・採算管理の統括</t>
-  </si>
-  <si>
-    <t xml:space="preserve">中期財務・人件費計画の策定</t>
-  </si>
-  <si>
-    <t xml:space="preserve">財務戦略・投資判断</t>
-  </si>
-  <si>
-    <t xml:space="preserve">広報・ブランディング</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PR</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">社内報・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SNS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">HP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の更新</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">社内・採用広報の企画作成</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">広報計画・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Corporate Site</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">管理</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">採用ブランディング・発信の統括</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ブランド戦略の策定</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ブランド・評判の責任者</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">IT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・情報セキュリティ</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">IT</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">アカウント・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">手配・一次対応</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">SaaS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ツールの運用管理</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">活用の企画・セキュリティ運用</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">社内</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">IT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・セキュリティ・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の統括</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">IT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">戦略とセキュリティ方針</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">IT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">ガバナンスの責任者</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">経営情報の収集・入力</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MBR</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の集計・資料作成</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分析・会議資料の品質担保</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MBR</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">運営・予実管理の統括</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">中期計画・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・会議体の設計</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">経営計画・経営会議を主導</t>
-  </si>
-  <si>
+      <t xml:space="preserve">出所：同ドラフト </t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">出所：同ドラフト </t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">v02</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">v02</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">「コンピテンシー定義（期待水準の要約）」。全文は</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">「専門領域スキル」。機能名は</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Excel</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">HR</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の「</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・</t>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">02_</t>
     </r>
     <r>
       <rPr>
         <sz val="9"/>
         <color rgb="FF595959"/>
-        <rFont val="Meiryo UI"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FIN</t>
-    </r>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">コンピテンシー定義」を参照。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">専門領域</t>
+  </si>
+  <si>
+    <t xml:space="preserve">タイトルに付ける機能名（仮）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">入退社・勤怠・社保の手続</t>
+  </si>
+  <si>
+    <t xml:space="preserve">労務運用・評価の事務局</t>
+  </si>
+  <si>
+    <t xml:space="preserve">運用設計・規程改定の起案</t>
+  </si>
+  <si>
+    <t xml:space="preserve">評価・採用・育成の統括</t>
+  </si>
+  <si>
+    <t xml:space="preserve">要員計画・人事制度の設計</t>
+  </si>
+  <si>
+    <t xml:space="preserve">人事戦略・報酬原資の決定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">総務</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">備品・施設の依頼を処理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">総務運用・社内イベント運営</t>
+  </si>
+  <si>
+    <t xml:space="preserve">総務プロセス設計・ベンダー管理</t>
+  </si>
+  <si>
+    <t xml:space="preserve">総務・規程・監査対応の統括</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">BCP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・リスク管理方針の策定</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">リスク・コンプラ統制の責任者</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経理・財務</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経費精算・請求書のチェック</t>
+  </si>
+  <si>
+    <t xml:space="preserve">計数集計・本体経理との照合</t>
+  </si>
+  <si>
+    <t xml:space="preserve">月次決算・予実分析のリード</t>
+  </si>
+  <si>
+    <t xml:space="preserve">予算・予実・採算管理の統括</t>
+  </si>
+  <si>
+    <t xml:space="preserve">中期財務・人件費計画の策定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">財務戦略・投資判断</t>
+  </si>
+  <si>
+    <t xml:space="preserve">広報・ブランディング</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PR</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">社内報・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SNS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">HP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の更新</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">社内・採用広報の企画作成</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">広報計画・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Corporate Site</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">管理</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">採用ブランディング・発信の統括</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ブランド戦略の策定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ブランド・評判の責任者</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・情報セキュリティ</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">IT</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">アカウント・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">手配・一次対応</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SaaS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ツールの運用管理</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">活用の企画・セキュリティ運用</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">社内</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・セキュリティ・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の統括</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">戦略とセキュリティ方針</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ガバナンスの責任者</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">CP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">経営情報の収集・入力</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MBR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の集計・資料作成</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">KPI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分析・会議資料の品質担保</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MBR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">運営・予実管理の統括</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">中期計画・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">KPI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・会議体の設計</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">経営計画・経営会議を主導</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="9"/>
@@ -6568,7 +6519,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">以外は仮置き（</t>
+      <t xml:space="preserve">出所：同ドラフト </t>
     </r>
     <r>
       <rPr>
@@ -6578,7 +6529,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">GA</t>
+      <t xml:space="preserve">v02</t>
     </r>
     <r>
       <rPr>
@@ -6587,7 +6538,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">・</t>
+      <t xml:space="preserve">「専門領域スキル」。機能名は</t>
     </r>
     <r>
       <rPr>
@@ -6597,7 +6548,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">PR</t>
+      <t xml:space="preserve">HR</t>
     </r>
     <r>
       <rPr>
@@ -6616,7 +6567,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">IT</t>
+      <t xml:space="preserve">FIN</t>
     </r>
     <r>
       <rPr>
@@ -6625,7 +6576,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">・</t>
+      <t xml:space="preserve">以外は仮置き（</t>
     </r>
     <r>
       <rPr>
@@ -6635,7 +6586,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">CP</t>
+      <t xml:space="preserve">GA</t>
     </r>
     <r>
       <rPr>
@@ -6644,6 +6595,63 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Meiryo UI"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">）。</t>
     </r>
   </si>
@@ -6669,9 +6677,6 @@
       </rPr>
       <t xml:space="preserve">区分</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">財務</t>
   </si>
 </sst>
 </file>
@@ -8299,7 +8304,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A51:A54" type="list">
-      <formula1>マスタ!$A$45:$A$46</formula1>
+      <formula1>マスタ!$A$45:$A$45</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -9213,7 +9218,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A51:A54" type="list">
-      <formula1>マスタ!$A$45:$A$46</formula1>
+      <formula1>マスタ!$A$45:$A$45</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -10155,7 +10160,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A51:A54" type="list">
-      <formula1>マスタ!$A$45:$A$46</formula1>
+      <formula1>マスタ!$A$45:$A$45</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -10175,7 +10180,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -10381,7 +10386,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>147</v>
       </c>
@@ -10407,15 +10412,15 @@
         <v>254</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="J8" s="34" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10709,7 +10714,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="42.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10717,22 +10722,22 @@
         <v>52</v>
       </c>
       <c r="B23" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="C23" s="27" t="s">
         <v>258</v>
       </c>
-      <c r="C23" s="27" t="s">
+      <c r="D23" s="27" t="s">
         <v>259</v>
       </c>
-      <c r="D23" s="27" t="s">
+      <c r="E23" s="27" t="s">
         <v>260</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="F23" s="27" t="s">
         <v>261</v>
       </c>
-      <c r="F23" s="27" t="s">
+      <c r="G23" s="27" t="s">
         <v>262</v>
-      </c>
-      <c r="G23" s="27" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10740,22 +10745,22 @@
         <v>59</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>268</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10763,22 +10768,22 @@
         <v>60</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>274</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10786,22 +10791,22 @@
         <v>61</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>280</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10809,22 +10814,22 @@
         <v>62</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10832,22 +10837,22 @@
         <v>63</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>290</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10855,22 +10860,22 @@
         <v>65</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="G29" s="4" t="s">
         <v>296</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10878,22 +10883,22 @@
         <v>66</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="G30" s="3" t="s">
         <v>302</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10901,22 +10906,22 @@
         <v>68</v>
       </c>
       <c r="B31" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="D31" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="G31" s="3" t="s">
         <v>308</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10924,35 +10929,35 @@
         <v>69</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="E32" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="F32" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="G32" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="B35" s="17" t="s">
         <v>317</v>
-      </c>
-      <c r="B35" s="17" t="s">
-        <v>318</v>
       </c>
       <c r="C35" s="27" t="s">
         <v>96</v>
@@ -10978,129 +10983,129 @@
         <v>97</v>
       </c>
       <c r="B36" s="37" t="s">
+        <v>318</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="H36" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="B37" s="37" t="s">
         <v>326</v>
       </c>
-      <c r="B37" s="37" t="s">
+      <c r="C37" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="D37" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="F37" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="G37" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="H37" s="3" t="s">
         <v>332</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="B38" s="37" t="s">
         <v>334</v>
       </c>
-      <c r="B38" s="37" t="s">
+      <c r="C38" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="D38" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="E38" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="F38" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="G38" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="G38" s="3" t="s">
+      <c r="H38" s="3" t="s">
         <v>340</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B39" s="37" t="s">
         <v>342</v>
       </c>
-      <c r="B39" s="37" t="s">
+      <c r="C39" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="D39" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="E39" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="F39" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="G39" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="H39" s="3" t="s">
         <v>348</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B40" s="37" t="s">
         <v>350</v>
       </c>
-      <c r="B40" s="37" t="s">
+      <c r="C40" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="D40" s="4" t="s">
         <v>352</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="E40" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="F40" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="4" t="s">
         <v>355</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>356</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="29.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11108,45 +11113,40 @@
         <v>145</v>
       </c>
       <c r="B41" s="37" t="s">
+        <v>357</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="D41" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="E41" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="E41" s="4" t="s">
+      <c r="F41" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="G41" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="G41" s="3" t="s">
+      <c r="H41" s="3" t="s">
         <v>363</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="38" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="39" t="s">
         <v>190</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="39" t="s">
-        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>